<commit_message>
include aaa-indie in standardized_coefficients.py and .csv
</commit_message>
<xml_diff>
--- a/output/coefficients/standardized/standardized_JP.xlsx
+++ b/output/coefficients/standardized/standardized_JP.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,18 +460,18 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1269</v>
+        <v>0.1393</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0056</v>
+        <v>0.0058</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>22.7903</v>
+        <v>24.0928</v>
       </c>
       <c r="G2" t="n">
-        <v>5.719919393903775e-115</v>
+        <v>2.973277728886143e-128</v>
       </c>
     </row>
     <row r="3">
@@ -481,22 +481,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0127</v>
+        <v>0.0116</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0026</v>
+        <v>0.0025</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0738</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0149</v>
+        <v>0.0147</v>
       </c>
       <c r="F3" t="n">
-        <v>4.9405</v>
+        <v>4.6011</v>
       </c>
       <c r="G3" t="n">
-        <v>7.792589020641442e-07</v>
+        <v>4.201972236188619e-06</v>
       </c>
     </row>
     <row r="4">
@@ -506,22 +506,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.0178</v>
+        <v>-0.0134</v>
       </c>
       <c r="C4" t="n">
         <v>0.0037</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.07489999999999999</v>
+        <v>-0.0565</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0158</v>
+        <v>0.0156</v>
       </c>
       <c r="F4" t="n">
-        <v>-4.7546</v>
+        <v>-3.6109</v>
       </c>
       <c r="G4" t="n">
-        <v>1.988349022704924e-06</v>
+        <v>0.0003051525889843639</v>
       </c>
     </row>
     <row r="5">
@@ -531,22 +531,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.0044</v>
+        <v>-0.0043</v>
       </c>
       <c r="C5" t="n">
         <v>0.0004</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.2003</v>
+        <v>-0.1965</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0161</v>
+        <v>0.016</v>
       </c>
       <c r="F5" t="n">
-        <v>-12.4537</v>
+        <v>-12.2809</v>
       </c>
       <c r="G5" t="n">
-        <v>1.334427727785046e-35</v>
+        <v>1.147278220178956e-34</v>
       </c>
     </row>
     <row r="6">
@@ -556,22 +556,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.0207</v>
+        <v>-0.0276</v>
       </c>
       <c r="C6" t="n">
-        <v>0.005</v>
+        <v>0.0051</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.07480000000000001</v>
+        <v>-0.0999</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0182</v>
+        <v>0.0183</v>
       </c>
       <c r="F6" t="n">
-        <v>-4.1141</v>
+        <v>-5.4657</v>
       </c>
       <c r="G6" t="n">
-        <v>3.886357916280625e-05</v>
+        <v>4.610764476576635e-08</v>
       </c>
     </row>
     <row r="7">
@@ -581,22 +581,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0014</v>
+        <v>-0.0145</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0068</v>
+        <v>0.007</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0039</v>
+        <v>-0.0416</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0197</v>
+        <v>0.0202</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1983</v>
+        <v>-2.0558</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8427909080393092</v>
+        <v>0.03979982084358254</v>
       </c>
     </row>
     <row r="8">
@@ -606,22 +606,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.0278</v>
+        <v>-0.0277</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0059</v>
+        <v>0.0058</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0828</v>
+        <v>-0.0824</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0175</v>
+        <v>0.0173</v>
       </c>
       <c r="F8" t="n">
-        <v>-4.7231</v>
+        <v>-4.7519</v>
       </c>
       <c r="G8" t="n">
-        <v>2.322951006754869e-06</v>
+        <v>2.015223998359697e-06</v>
       </c>
     </row>
     <row r="9">
@@ -631,22 +631,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.0566</v>
+        <v>-0.0495</v>
       </c>
       <c r="C9" t="n">
         <v>0.0044</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.1982</v>
+        <v>-0.1734</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0154</v>
+        <v>0.0153</v>
       </c>
       <c r="F9" t="n">
-        <v>-12.8561</v>
+        <v>-11.3685</v>
       </c>
       <c r="G9" t="n">
-        <v>7.949098793573911e-38</v>
+        <v>6.003318545909891e-30</v>
       </c>
     </row>
     <row r="10">
@@ -656,22 +656,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.0371</v>
+        <v>-0.0439</v>
       </c>
       <c r="C10" t="n">
         <v>0.006</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0905</v>
+        <v>-0.107</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0146</v>
+        <v>0.0147</v>
       </c>
       <c r="F10" t="n">
-        <v>-6.1938</v>
+        <v>-7.2786</v>
       </c>
       <c r="G10" t="n">
-        <v>5.871625820920273e-10</v>
+        <v>3.37288044545696e-13</v>
       </c>
     </row>
     <row r="11">
@@ -681,22 +681,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.0679</v>
+        <v>-0.0709</v>
       </c>
       <c r="C11" t="n">
         <v>0.0061</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.1229</v>
+        <v>-0.1281</v>
       </c>
       <c r="E11" t="n">
         <v>0.011</v>
       </c>
       <c r="F11" t="n">
-        <v>-11.1725</v>
+        <v>-11.6207</v>
       </c>
       <c r="G11" t="n">
-        <v>5.556307084838132e-29</v>
+        <v>3.233128502358928e-31</v>
       </c>
     </row>
     <row r="12">
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.0342</v>
+        <v>-0.0344</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0073</v>
+        <v>0.0072</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0728</v>
+        <v>-0.0732</v>
       </c>
       <c r="E12" t="n">
         <v>0.0154</v>
       </c>
       <c r="F12" t="n">
-        <v>-4.715</v>
+        <v>-4.7625</v>
       </c>
       <c r="G12" t="n">
-        <v>2.417144481668843e-06</v>
+        <v>1.91211945963566e-06</v>
       </c>
     </row>
     <row r="13">
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.0336</v>
+        <v>-0.0439</v>
       </c>
       <c r="C13" t="n">
         <v>0.0091</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0539</v>
+        <v>-0.0704</v>
       </c>
       <c r="E13" t="n">
         <v>0.0146</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.6891</v>
+        <v>-4.8254</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0002250604045411201</v>
+        <v>1.397440453692042e-06</v>
       </c>
     </row>
     <row r="14">
@@ -756,22 +756,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.0282</v>
+        <v>-0.0294</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0061</v>
+        <v>0.006</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.068</v>
+        <v>-0.0711</v>
       </c>
       <c r="E14" t="n">
         <v>0.0146</v>
       </c>
       <c r="F14" t="n">
-        <v>-4.6432</v>
+        <v>-4.8768</v>
       </c>
       <c r="G14" t="n">
-        <v>3.429742796471264e-06</v>
+        <v>1.078040353427481e-06</v>
       </c>
     </row>
     <row r="15">
@@ -781,22 +781,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.009299999999999999</v>
+        <v>-0.0156</v>
       </c>
       <c r="C15" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0177</v>
+        <v>-0.0295</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0159</v>
+        <v>0.0161</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.1158</v>
+        <v>-1.8283</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2644871290746181</v>
+        <v>0.06750116419621574</v>
       </c>
     </row>
     <row r="16">
@@ -806,22 +806,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.034</v>
+        <v>-0.0412</v>
       </c>
       <c r="C16" t="n">
         <v>0.0086</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0477</v>
+        <v>-0.0577</v>
       </c>
       <c r="E16" t="n">
         <v>0.012</v>
       </c>
       <c r="F16" t="n">
-        <v>-3.9727</v>
+        <v>-4.7911</v>
       </c>
       <c r="G16" t="n">
-        <v>7.105818977226174e-05</v>
+        <v>1.658427009483529e-06</v>
       </c>
     </row>
     <row r="17">
@@ -831,22 +831,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.0315</v>
+        <v>-0.042</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0069</v>
+        <v>0.007</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.0401</v>
+        <v>-0.0535</v>
       </c>
       <c r="E17" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0089</v>
       </c>
       <c r="F17" t="n">
-        <v>-4.5574</v>
+        <v>-6.0261</v>
       </c>
       <c r="G17" t="n">
-        <v>5.178697854291059e-06</v>
+        <v>1.679855939870908e-09</v>
       </c>
     </row>
     <row r="18">
@@ -856,22 +856,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.049</v>
+        <v>-0.0375</v>
       </c>
       <c r="C18" t="n">
         <v>0.0044</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0888</v>
+        <v>-0.068</v>
       </c>
       <c r="E18" t="n">
         <v>0.008</v>
       </c>
       <c r="F18" t="n">
-        <v>-11.1412</v>
+        <v>-8.5556</v>
       </c>
       <c r="G18" t="n">
-        <v>7.906114396722562e-29</v>
+        <v>1.172793169560562e-17</v>
       </c>
     </row>
     <row r="19">
@@ -881,22 +881,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0244</v>
+        <v>0.0181</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0166</v>
+        <v>0.0161</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0229</v>
+        <v>0.0169</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0155</v>
+        <v>0.0151</v>
       </c>
       <c r="F19" t="n">
-        <v>1.4746</v>
+        <v>1.1194</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1403202084202728</v>
+        <v>0.2629609945769958</v>
       </c>
     </row>
     <row r="20">
@@ -906,22 +906,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.029</v>
+        <v>0.0158</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0235</v>
+        <v>0.0245</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0193</v>
+        <v>0.0105</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0156</v>
+        <v>0.0163</v>
       </c>
       <c r="F20" t="n">
-        <v>1.234</v>
+        <v>0.6433</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2171959761181209</v>
+        <v>0.5200393055702741</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.0041</v>
+        <v>-0.0086</v>
       </c>
       <c r="C21" t="n">
-        <v>0.0166</v>
+        <v>0.0162</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.003</v>
+        <v>-0.0065</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0124</v>
+        <v>0.0121</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2449</v>
+        <v>-0.5315</v>
       </c>
       <c r="G21" t="n">
-        <v>0.806509111750946</v>
+        <v>0.5950808586216669</v>
       </c>
     </row>
     <row r="22">
@@ -959,19 +959,19 @@
         <v>0.0023</v>
       </c>
       <c r="C22" t="n">
-        <v>0.0038</v>
+        <v>0.0037</v>
       </c>
       <c r="D22" t="n">
         <v>0.009900000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0162</v>
+        <v>0.016</v>
       </c>
       <c r="F22" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.6157</v>
       </c>
       <c r="G22" t="n">
-        <v>0.5416244107718886</v>
+        <v>0.5381087955485305</v>
       </c>
     </row>
     <row r="23">
@@ -981,22 +981,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.0242</v>
+        <v>-0.0266</v>
       </c>
       <c r="C23" t="n">
         <v>0.0053</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0589</v>
+        <v>-0.065</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0129</v>
+        <v>0.013</v>
       </c>
       <c r="F23" t="n">
-        <v>-4.5519</v>
+        <v>-4.9926</v>
       </c>
       <c r="G23" t="n">
-        <v>5.316557525235557e-06</v>
+        <v>5.955884042550342e-07</v>
       </c>
     </row>
     <row r="24">
@@ -1006,22 +1006,22 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.0713</v>
+        <v>-0.07190000000000001</v>
       </c>
       <c r="C24" t="n">
         <v>0.0034</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.2003</v>
+        <v>-0.2017</v>
       </c>
       <c r="E24" t="n">
         <v>0.009599999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>-20.9511</v>
+        <v>-20.9874</v>
       </c>
       <c r="G24" t="n">
-        <v>1.833481854511251e-97</v>
+        <v>8.549389740776044e-98</v>
       </c>
     </row>
     <row r="25">
@@ -1031,22 +1031,97 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.0178</v>
+        <v>-0.013</v>
       </c>
       <c r="C25" t="n">
-        <v>0.003</v>
+        <v>0.0029</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.07630000000000001</v>
+        <v>-0.0557</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0127</v>
+        <v>0.0125</v>
       </c>
       <c r="F25" t="n">
-        <v>-5.9922</v>
+        <v>-4.4549</v>
       </c>
       <c r="G25" t="n">
-        <v>2.069937966897287e-09</v>
+        <v>8.392923020292335e-06</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>d_aa</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-0.0306</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.1157</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0124</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-9.331</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1.048921794262594e-20</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d_indie</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>-0.0367</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.0926</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-9.7531</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1.78922769219574e-22</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>d_unknown</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>-0.0375</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.141</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-11.4551</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2.21591782514193e-30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>